<commit_message>
+ final review, waiting for changes in business exception
</commit_message>
<xml_diff>
--- a/Nubank_Case_Performer/Data/Config.xlsx
+++ b/Nubank_Case_Performer/Data/Config.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vinic\Documents\UiPath\Nubank_Case_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vinic\Documents\StevanBOT_Git\Nubank_Case_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52F86B81-B28A-460D-A737-B5F66E7113D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B19936C-32AE-4197-ADD0-4F4F567E829B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="73">
   <si>
     <t>Name</t>
   </si>
@@ -243,13 +243,19 @@
   </si>
   <si>
     <t>Errors_Filepath</t>
+  </si>
+  <si>
+    <t>Filepath_Temp</t>
+  </si>
+  <si>
+    <t>Temp_Filepath</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -300,6 +306,11 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -321,7 +332,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -338,6 +349,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3033,7 +3045,14 @@
         <v>69</v>
       </c>
     </row>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="12" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>71</v>
+      </c>
+    </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="15" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>